<commit_message>
Arbeitsmappe: drei Systeme vorrecherchiert
lexoffice/Lexware Office, sevdesk und easybill eingetragen. Weisse
Zellen sind belegt, gelbe bleiben offen, Quellen in Spalte O.

Wichtigster Befund, woertlich aus der Lexware-Hilfe belegt: Lexware
Office unterstuetzt Paragraf 13b Bauleistungen aktuell NICHT im
XRechnung- oder ZUGFeRD-Format, diese Rechnungen sind dort nur als PDF
moeglich. Bis 2027/2028 ist PDF noch zulaessig, danach nicht mehr.
Fuer Baubetriebe auf lexoffice ist das kein Einrichtungsauftrag,
sondern ein Gespraech ueber einen Systemwechsel.

Angaben zu sevdesk stammen aus Drittquellen und sind als solche
markiert; die Paragraf-13b-Faehigkeit von sevdesk und easybill ist
offen und muss vor dem ersten Kunden geprueft werden.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECQV3LX17FPwV9aCb3VGtx
</commit_message>
<xml_diff>
--- a/erechnung/E-Rechnung_Arbeitsmappe.xlsx
+++ b/erechnung/E-Rechnung_Arbeitsmappe.xlsx
@@ -128,7 +128,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -148,6 +148,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F1EC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -221,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -288,6 +293,16 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -688,6 +703,13 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="29" t="inlineStr">
+        <is>
+          <t>Drei Zeilen sind vorrecherchiert (04.09.2026). Weiss = belegt. Gelb = noch offen. Quellen stehen in Spalte O.</t>
+        </is>
+      </c>
+    </row>
     <row r="4" ht="26" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -847,7 +869,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
+    <row r="7" ht="86" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>lexoffice / Lexware Office</t>
@@ -863,20 +885,66 @@
           <t>Kern</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="9" t="n"/>
-      <c r="I7" s="9" t="n"/>
-      <c r="J7" s="9" t="n"/>
-      <c r="K7" s="9" t="n"/>
-      <c r="L7" s="9" t="n"/>
-      <c r="M7" s="9" t="n"/>
-      <c r="N7" s="9" t="n"/>
-      <c r="O7" s="9" t="n"/>
-    </row>
-    <row r="8" ht="30" customHeight="1">
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>04.09.2026</t>
+        </is>
+      </c>
+      <c r="E7" s="30" t="inlineStr">
+        <is>
+          <t>ab Paket M</t>
+        </is>
+      </c>
+      <c r="F7" s="30" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G7" s="30" t="inlineStr">
+        <is>
+          <t>XRechnung + ZUGFeRD</t>
+        </is>
+      </c>
+      <c r="H7" s="30" t="inlineStr">
+        <is>
+          <t>Einstellungen (Zahnrad) &gt; E-Rechnung &gt; „E-Rechnung erstellen“. Admin-Rechte noetig.</t>
+        </is>
+      </c>
+      <c r="I7" s="30" t="inlineStr">
+        <is>
+          <t>Kontakt muss als „Firma“ angelegt sein — an Privatpersonen ist keine E-Rechnung moeglich. Bei Behoerden zusaetzlich Leitweg-ID und Lieferantennummer.</t>
+        </is>
+      </c>
+      <c r="J7" s="31" t="inlineStr">
+        <is>
+          <t>NEIN — nur als PDF! Rechnungsart oben rechts „§13b – Bauleistung“, vorher im Kundenstamm &gt; Steuerangaben Haekchen „Steuerfreie Rechnungen erlauben“. Lexware selbst: §13b wird aktuell NICHT im XRechnung- oder ZUGFeRD-Format unterstuetzt.</t>
+        </is>
+      </c>
+      <c r="K7" s="30" t="inlineStr">
+        <is>
+          <t>Kundenstamm, Pflichtfeld bei Behoerden</t>
+        </is>
+      </c>
+      <c r="L7" s="30" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="M7" s="31" t="inlineStr">
+        <is>
+          <t>GROESSTER PUNKT: Baubetriebe mit §13b koennen mit Lexware Office ab 2028 keine gueltige E-Rechnung stellen. Bis 2027/2028 ist PDF noch zulaessig, danach nicht mehr. Das ist kein Einrichtungsauftrag, sondern ein Gespraech ueber einen Systemwechsel.</t>
+        </is>
+      </c>
+      <c r="N7" s="30" t="n">
+        <v>2</v>
+      </c>
+      <c r="O7" s="30" t="inlineStr">
+        <is>
+          <t>help.lexware.de/de-form/articles/547939 und /547981</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="86" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>sevdesk</t>
@@ -892,18 +960,62 @@
           <t>Kern</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
-      <c r="J8" s="9" t="n"/>
-      <c r="K8" s="9" t="n"/>
-      <c r="L8" s="9" t="n"/>
-      <c r="M8" s="9" t="n"/>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>04.09.2026</t>
+        </is>
+      </c>
+      <c r="E8" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="F8" s="30" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G8" s="30" t="inlineStr">
+        <is>
+          <t>XRechnung (UBL) + ZUGFeRD 2.1 / 2.2</t>
+        </is>
+      </c>
+      <c r="H8" s="30" t="inlineStr">
+        <is>
+          <t>Einstellungen &gt; Rechnungen: Standardformat auf XRechnung oder ZUGFeRD setzen. QUELLE DRITTANBIETER — in der sevdesk-Hilfe gegenpruefen.</t>
+        </is>
+      </c>
+      <c r="I8" s="30" t="inlineStr">
+        <is>
+          <t>USt-IdNr., Bankverbindung, Handelsregisternummer unter Einstellungen &gt; Unternehmen</t>
+        </is>
+      </c>
+      <c r="J8" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen — — unbedingt selbst pruefen, siehe Lexware-Zeile</t>
+        </is>
+      </c>
+      <c r="K8" s="30" t="inlineStr">
+        <is>
+          <t>im Kontaktdatensatz des Empfaengers</t>
+        </is>
+      </c>
+      <c r="L8" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="M8" s="30" t="inlineStr">
+        <is>
+          <t>Angaben stammen aus Drittquellen, nicht aus der Herstellerhilfe. Vor dem ersten Kunden verifizieren.</t>
+        </is>
+      </c>
       <c r="N8" s="9" t="n"/>
-      <c r="O8" s="9" t="n"/>
+      <c r="O8" s="30" t="inlineStr">
+        <is>
+          <t>sevdesk.de/funktion-e-rechnung (Herstellerhilfe noch pruefen)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
@@ -934,7 +1046,7 @@
       <c r="N9" s="9" t="n"/>
       <c r="O9" s="9" t="n"/>
     </row>
-    <row r="10" ht="30" customHeight="1">
+    <row r="10" ht="86" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>easybill</t>
@@ -950,18 +1062,62 @@
           <t>Kern</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="9" t="n"/>
-      <c r="J10" s="9" t="n"/>
-      <c r="K10" s="9" t="n"/>
-      <c r="L10" s="9" t="n"/>
-      <c r="M10" s="9" t="n"/>
+      <c r="D10" s="30" t="inlineStr">
+        <is>
+          <t>04.09.2026</t>
+        </is>
+      </c>
+      <c r="E10" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G10" s="30" t="inlineStr">
+        <is>
+          <t>XRechnung 3.0.2 + ZUGFeRD</t>
+        </is>
+      </c>
+      <c r="H10" s="30" t="inlineStr">
+        <is>
+          <t>Kunde oeffnen &gt; Bearbeiten &gt; Einstellungen &gt; Dokumentformat fuer den Versand. Wird JE KUNDE eingestellt, nicht zentral.</t>
+        </is>
+      </c>
+      <c r="I10" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="J10" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen — — unbedingt selbst pruefen</t>
+        </is>
+      </c>
+      <c r="K10" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="L10" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="M10" s="30" t="inlineStr">
+        <is>
+          <t>Format je Kunde statt global — bei vielen Bestandskunden entsteht Mehraufwand. Hersteller empfiehlt, ZUGFeRD als Standard fuer alle Vorlagen zu setzen.</t>
+        </is>
+      </c>
       <c r="N10" s="9" t="n"/>
-      <c r="O10" s="9" t="n"/>
+      <c r="O10" s="30" t="inlineStr">
+        <is>
+          <t>support.easybill.de/hc/de/articles/13571616499228 und /14557057264412</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
@@ -1448,9 +1604,10 @@
       <c r="O26" s="13" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:O1"/>
     <mergeCell ref="A4:O4"/>
+    <mergeCell ref="A3:O3"/>
     <mergeCell ref="A2:O2"/>
   </mergeCells>
   <dataValidations count="2">
@@ -1890,12 +2047,12 @@
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A18:E18"/>
     <mergeCell ref="A24:E24"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A14:E14"/>
+    <mergeCell ref="A18:E18"/>
     <mergeCell ref="A9:E9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Arbeitsmappe: alle neun Kernsysteme bearbeitet, Paragraf 13b praezisiert
Kernliste durchgearbeitet: 53 Zellen belegt, 46 bleiben offen und sind
als solche markiert. Belegt ist, was sich an einer Quelle nachweisen
liess; geraten wurde nichts.

Fehlerkatalog Rang 2 traegt jetzt die exakte Vorgabe: Steuerkategorie
AE, Steuersatz 0, Befreiungsgrund-Code VATEX-EU-AE und der
Befreiungstext zur Steuerschuldnerschaft des Leistungsempfaengers.

Blatt 4 ergaenzt um eine ehrliche Einordnung des eigenen Lesers:
kostenlose Betrachter existieren bereits (Quba, RIB, Mustang). Der
Leser ist kein Produkt, sondern ein Gespraechsoeffner.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECQV3LX17FPwV9aCb3VGtx
</commit_message>
<xml_diff>
--- a/erechnung/E-Rechnung_Arbeitsmappe.xlsx
+++ b/erechnung/E-Rechnung_Arbeitsmappe.xlsx
@@ -226,7 +226,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -302,6 +302,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1017,7 +1024,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="74" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>WISO Mein Buero</t>
@@ -1033,18 +1040,62 @@
           <t>Kern</t>
         </is>
       </c>
-      <c r="D9" s="9" t="n"/>
-      <c r="E9" s="9" t="n"/>
-      <c r="F9" s="9" t="n"/>
-      <c r="G9" s="9" t="n"/>
-      <c r="H9" s="9" t="n"/>
-      <c r="I9" s="9" t="n"/>
-      <c r="J9" s="9" t="n"/>
-      <c r="K9" s="9" t="n"/>
-      <c r="L9" s="9" t="n"/>
-      <c r="M9" s="9" t="n"/>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>04.09.2026</t>
+        </is>
+      </c>
+      <c r="E9" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="F9" s="30" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G9" s="30" t="inlineStr">
+        <is>
+          <t>ZUGFeRD automatisch, XRechnung als XML-Download</t>
+        </is>
+      </c>
+      <c r="H9" s="30" t="inlineStr">
+        <is>
+          <t>Einstellungen &gt; Meine Firma &gt; E-Rechnungen</t>
+        </is>
+      </c>
+      <c r="I9" s="30" t="inlineStr">
+        <is>
+          <t>Bankverbindung und Kontaktdaten pflicht. Nur B2B — an Privatkunden keine E-Rechnung.</t>
+        </is>
+      </c>
+      <c r="J9" s="33" t="inlineStr">
+        <is>
+          <t>— noch offen — — WICHTIGSTE FRAGE, siehe Blatt 3</t>
+        </is>
+      </c>
+      <c r="K9" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="L9" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="M9" s="30" t="inlineStr">
+        <is>
+          <t>Jede Rechnung wird automatisch als ZUGFeRD erzeugt; die XRechnung-XML muss man nach dem Abschliessen separat herunterladen. Desktop- und Web-Version unterscheiden sich — vorher klaeren, welche der Kunde hat.</t>
+        </is>
+      </c>
       <c r="N9" s="9" t="n"/>
-      <c r="O9" s="9" t="n"/>
+      <c r="O9" s="30" t="inlineStr">
+        <is>
+          <t>handbuch.meinbuero.de/mbr-e-rechnung/e-rechnung-erstellen</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="86" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
@@ -1119,7 +1170,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
+    <row r="11" ht="74" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t>FastBill</t>
@@ -1135,20 +1186,64 @@
           <t>Kern</t>
         </is>
       </c>
-      <c r="D11" s="9" t="n"/>
-      <c r="E11" s="9" t="n"/>
-      <c r="F11" s="9" t="n"/>
-      <c r="G11" s="9" t="n"/>
-      <c r="H11" s="9" t="n"/>
-      <c r="I11" s="9" t="n"/>
-      <c r="J11" s="9" t="n"/>
-      <c r="K11" s="9" t="n"/>
-      <c r="L11" s="9" t="n"/>
-      <c r="M11" s="9" t="n"/>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>04.09.2026</t>
+        </is>
+      </c>
+      <c r="E11" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G11" s="30" t="inlineStr">
+        <is>
+          <t>XRechnung + ZUGFeRD</t>
+        </is>
+      </c>
+      <c r="H11" s="30" t="inlineStr">
+        <is>
+          <t>E-Rechnungs-Option aktivieren, dann wird bei „Rechnung erstellen“ automatisch beides erzeugt</t>
+        </is>
+      </c>
+      <c r="I11" s="30" t="inlineStr">
+        <is>
+          <t>Alle Pflichtangaben muessen gefuellt sein, sonst wird keine E-Rechnung erzeugt — welche genau: offen</t>
+        </is>
+      </c>
+      <c r="J11" s="33" t="inlineStr">
+        <is>
+          <t>— noch offen — — WICHTIGSTE FRAGE, siehe Blatt 3</t>
+        </is>
+      </c>
+      <c r="K11" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="L11" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="M11" s="30" t="inlineStr">
+        <is>
+          <t>Erzeugt ZUGFeRD und XRechnung gleichzeitig. Erzeugt sie nur, wenn alle Pflichtfelder gefuellt sind — sonst still kein E-Rechnungs-Ergebnis. Genau hinsehen.</t>
+        </is>
+      </c>
       <c r="N11" s="9" t="n"/>
-      <c r="O11" s="9" t="n"/>
-    </row>
-    <row r="12" ht="30" customHeight="1">
+      <c r="O11" s="30" t="inlineStr">
+        <is>
+          <t>support.fastbill.com/hc/de/articles/22209126147484</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="74" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Billomat</t>
@@ -1164,20 +1259,64 @@
           <t>Kern</t>
         </is>
       </c>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="n"/>
-      <c r="J12" s="9" t="n"/>
-      <c r="K12" s="9" t="n"/>
-      <c r="L12" s="9" t="n"/>
-      <c r="M12" s="9" t="n"/>
+      <c r="D12" s="30" t="inlineStr">
+        <is>
+          <t>04.09.2026</t>
+        </is>
+      </c>
+      <c r="E12" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="G12" s="30" t="inlineStr">
+        <is>
+          <t>XRechnung + ZUGFeRD</t>
+        </is>
+      </c>
+      <c r="H12" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="I12" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="J12" s="33" t="inlineStr">
+        <is>
+          <t>— noch offen — — WICHTIGSTE FRAGE, siehe Blatt 3</t>
+        </is>
+      </c>
+      <c r="K12" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="L12" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="M12" s="30" t="inlineStr">
+        <is>
+          <t>Unterstuetzung bestaetigt, Einrichtungsdetails noch nicht recherchiert.</t>
+        </is>
+      </c>
       <c r="N12" s="9" t="n"/>
-      <c r="O12" s="9" t="n"/>
-    </row>
-    <row r="13" ht="30" customHeight="1">
+      <c r="O12" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="74" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Papierkram</t>
@@ -1193,20 +1332,64 @@
           <t>Kern</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
-      <c r="G13" s="9" t="n"/>
-      <c r="H13" s="9" t="n"/>
-      <c r="I13" s="9" t="n"/>
-      <c r="J13" s="9" t="n"/>
-      <c r="K13" s="9" t="n"/>
-      <c r="L13" s="9" t="n"/>
-      <c r="M13" s="9" t="n"/>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>04.09.2026</t>
+        </is>
+      </c>
+      <c r="E13" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="F13" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="G13" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="H13" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="I13" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="J13" s="33" t="inlineStr">
+        <is>
+          <t>— noch offen — — WICHTIGSTE FRAGE, siehe Blatt 3</t>
+        </is>
+      </c>
+      <c r="K13" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="L13" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="M13" s="30" t="inlineStr">
+        <is>
+          <t>Nichts Belastbares gefunden. Herstellerhilfe direkt aufrufen.</t>
+        </is>
+      </c>
       <c r="N13" s="9" t="n"/>
-      <c r="O13" s="9" t="n"/>
-    </row>
-    <row r="14" ht="30" customHeight="1">
+      <c r="O13" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="74" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t>SumUp Rechnungen</t>
@@ -1222,20 +1405,64 @@
           <t>Kern</t>
         </is>
       </c>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="9" t="n"/>
-      <c r="G14" s="9" t="n"/>
-      <c r="H14" s="9" t="n"/>
-      <c r="I14" s="9" t="n"/>
-      <c r="J14" s="9" t="n"/>
-      <c r="K14" s="9" t="n"/>
-      <c r="L14" s="9" t="n"/>
-      <c r="M14" s="9" t="n"/>
+      <c r="D14" s="30" t="inlineStr">
+        <is>
+          <t>04.09.2026</t>
+        </is>
+      </c>
+      <c r="E14" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="F14" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="G14" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="H14" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="I14" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="J14" s="33" t="inlineStr">
+        <is>
+          <t>— noch offen — — WICHTIGSTE FRAGE, siehe Blatt 3</t>
+        </is>
+      </c>
+      <c r="K14" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="L14" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="M14" s="30" t="inlineStr">
+        <is>
+          <t>Nichts Belastbares gefunden. Eher Kleinstgewerbe — pruefen, ob die Zielgruppe ueberhaupt zahlt.</t>
+        </is>
+      </c>
       <c r="N14" s="9" t="n"/>
-      <c r="O14" s="9" t="n"/>
-    </row>
-    <row r="15" ht="30" customHeight="1">
+      <c r="O14" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="74" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Collmex</t>
@@ -1251,18 +1478,62 @@
           <t>Kern</t>
         </is>
       </c>
-      <c r="D15" s="9" t="n"/>
-      <c r="E15" s="9" t="n"/>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="9" t="n"/>
-      <c r="H15" s="9" t="n"/>
-      <c r="I15" s="9" t="n"/>
-      <c r="J15" s="9" t="n"/>
-      <c r="K15" s="9" t="n"/>
-      <c r="L15" s="9" t="n"/>
-      <c r="M15" s="9" t="n"/>
+      <c r="D15" s="30" t="inlineStr">
+        <is>
+          <t>04.09.2026</t>
+        </is>
+      </c>
+      <c r="E15" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="G15" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="H15" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="I15" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="J15" s="33" t="inlineStr">
+        <is>
+          <t>— noch offen — — WICHTIGSTE FRAGE, siehe Blatt 3</t>
+        </is>
+      </c>
+      <c r="K15" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="L15" s="32" t="inlineStr">
+        <is>
+          <t>— noch offen —</t>
+        </is>
+      </c>
+      <c r="M15" s="30" t="inlineStr">
+        <is>
+          <t>Nichts Belastbares gefunden. Collmex ist im Handwerk verbreitet — lohnt eigene Recherche.</t>
+        </is>
+      </c>
       <c r="N15" s="9" t="n"/>
-      <c r="O15" s="9" t="n"/>
+      <c r="O15" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="10" t="inlineStr">
@@ -2139,7 +2410,7 @@
       </c>
       <c r="E5" s="9" t="n"/>
     </row>
-    <row r="6" ht="52" customHeight="1">
+    <row r="6" ht="90" customHeight="1">
       <c r="A6" s="22" t="inlineStr">
         <is>
           <t>2</t>
@@ -2155,9 +2426,9 @@
           <t>Steuersatz 0 %, aber Steuerkategorie steht auf „S“, oder der Hinweistext auf die Steuerschuldnerschaft des Leistungsempfaengers fehlt.</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>Kategorie „AE“ setzen und Befreiungsgrund als Text hinterlegen. Bei Baubetrieben der mit Abstand haeufigste Fehler — hier zuerst hinsehen. Ob § 13b gilt, entscheidet der Steuerberater, nicht du.</t>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Vier Angaben muessen zusammenpassen: Steuerkategorie „AE“, Steuersatz 0, Befreiungsgrund-Code „VATEX-EU-AE“ und der Befreiungstext „Steuerschuldnerschaft des Leistungsempfaengers“. Pruefen, ob die Software das automatisch setzt, sobald der Kunde als §13b-pflichtig markiert ist. ACHTUNG: Lexware Office kann §13b derzeit gar nicht als E-Rechnung ausgeben — siehe Blatt 1. Ob §13b gilt, entscheidet der Steuerberater, nicht du.</t>
         </is>
       </c>
       <c r="E6" s="9" t="n"/>
@@ -2361,7 +2632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2651,14 +2922,37 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="34" t="inlineStr">
+        <is>
+          <t>Zum Leser auf der Website — ehrlich eingeordnet</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="32" customHeight="1">
+      <c r="A27" s="35" t="inlineStr">
+        <is>
+          <t>•  Kostenlose E-Rechnungs-Betrachter gibt es bereits: Quba Viewer (vom Wirtschaftsministerium empfohlen), RIB Viewer, Mustang. Dein Leser ist technisch nichts Einzigartiges.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="35" t="inlineStr">
+        <is>
+          <t>•  Sein Wert liegt nicht in der Funktion, sondern darin, dass er auf DEINER Seite steht und dort das Gespraech eroeffnet. Verkaufe nie den Betrachter — verkaufe die Einrichtung.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A23:D23"/>
+    <mergeCell ref="A27:D27"/>
     <mergeCell ref="A22:D22"/>
     <mergeCell ref="A21:D21"/>
     <mergeCell ref="A24:D24"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A28:D28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
lexoffice §13b-Befund durch eigenen Test im Testkonto bestaetigt
Faruk hat heute im lexoffice-Testkonto Schritt fuer Schritt durchgespielt:
Kunde mit Haken 'Steuerfreie Rechnungen erlauben' angelegt, Rechnung wird
korrekt als 'Bauleistungen §13b' erkannt und zeigt den richtigen
Reverse-Charge-Text. Im Mailversand haengt trotzdem nur eine PDF, keine
XRechnung- oder ZUGFeRD-Datei. Der Befund von Lexware selbst (Stand 4.9.)
ist damit durch einen eigenen Test bestaetigt, nicht nur zitiert.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ECQV3LX17FPwV9aCb3VGtx
</commit_message>
<xml_diff>
--- a/erechnung/E-Rechnung_Arbeitsmappe.xlsx
+++ b/erechnung/E-Rechnung_Arbeitsmappe.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1 Systeme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2 Kundencheckliste" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="3 Fehlerkatalog" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="4 Angebot &amp; Regeln" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 Systeme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2 Kundencheckliste" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3 Fehlerkatalog" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4 Angebot &amp; Regeln" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -915,7 +915,7 @@
       </c>
       <c r="D7" s="30" t="inlineStr">
         <is>
-          <t>04.09.2026</t>
+          <t>04.09.2026 + eigener Test 11.09.2026</t>
         </is>
       </c>
       <c r="E7" s="30" t="inlineStr">
@@ -960,7 +960,7 @@
       </c>
       <c r="M7" s="31" t="inlineStr">
         <is>
-          <t>GROESSTER PUNKT: Baubetriebe mit §13b koennen mit Lexware Office ab 2028 keine gueltige E-Rechnung stellen. Bis 2027/2028 ist PDF noch zulaessig, danach nicht mehr. Das ist kein Einrichtungsauftrag, sondern ein Gespraech ueber einen Systemwechsel.</t>
+          <t>GROESSTER PUNKT: Baubetriebe mit §13b koennen mit Lexware Office ab 2028 keine gueltige E-Rechnung stellen. Bis 2027/2028 ist PDF noch zulaessig, danach nicht mehr. Das ist kein Einrichtungsauftrag, sondern ein Gespraech ueber einen Systemwechsel. EIGENER TEST am 11.09.2026 bestaetigt: Testkonto, Kunde mit Haken 'Steuerfreie Rechnungen erlauben', Rechnung wird korrekt als 'Bauleistungen §13b' erkannt und zeigt den richtigen Reverse-Charge-Text. Aber im Mailversand haengt trotzdem nur eine PDF, keine XRechnung/ZUGFeRD-Datei. Befund von Lexware selbst damit durch eigenen Test bestaetigt, nicht nur zitiert.</t>
         </is>
       </c>
       <c r="N7" s="30" t="n">

</xml_diff>